<commit_message>
Update RSVP & Multi-Function Check-In sheet (3 RSVPs, 0 Checked-In) [Sep 29, 10:21 AM]
</commit_message>
<xml_diff>
--- a/wedding-rsvps.xlsx
+++ b/wedding-rsvps.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="RSVP Responses" sheetId="1" r:id="rId1"/>
+    <sheet name="RSVP &amp; Check-Ins" sheetId="1" r:id="rId1"/>
     <sheet name="Summary &amp; Statistics" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
@@ -398,17 +398,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:O4"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="55.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="32.83203125" customWidth="1"/>
+    <col min="10" max="10" width="32.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="45.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,12 +437,30 @@
         <v>Total Guests Attending</v>
       </c>
       <c r="G1" t="str">
-        <v>Ceremonies Selected</v>
+        <v>Overall Check-In Status</v>
       </c>
       <c r="H1" t="str">
+        <v>Rukhsati (29 Oct) Check-In</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Ramada Reception (30 Oct) Check-In</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Radiant Reception (2 Nov) Check-In</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Latest Check-In Time</v>
+      </c>
+      <c r="L1" t="str">
+        <v>VIP Pass ID</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Invited Ceremonies</v>
+      </c>
+      <c r="N1" t="str">
         <v>Dietary Preferences</v>
       </c>
-      <c r="I1" t="str">
+      <c r="O1" t="str">
         <v>Heartfelt Duas &amp; Message</v>
       </c>
     </row>
@@ -445,43 +469,155 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-25T19:04:05.325Z</v>
+        <v>Sep 29, 2026, 10:18 AM</v>
       </c>
       <c r="C2" t="str">
-        <v>Tariq Ahmad</v>
+        <v>as</v>
       </c>
       <c r="D2" t="str">
-        <v>+91 98765 00000</v>
+        <v>6386687373</v>
       </c>
       <c r="E2" t="str">
         <v>Confirmed (Attending)</v>
       </c>
       <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>⏳ Awaiting Check-In</v>
+      </c>
+      <c r="H2" t="str">
+        <v>⏳ Awaiting Entry</v>
+      </c>
+      <c r="I2" t="str">
+        <v>⏳ Awaiting Entry</v>
+      </c>
+      <c r="J2" t="str">
+        <v>— Not Invited</v>
+      </c>
+      <c r="K2" t="str">
+        <v>—</v>
+      </c>
+      <c r="L2" t="str">
+        <v>—</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Rukhsati; Wedding Reception - Hotel Ramada</v>
+      </c>
+      <c r="N2" t="str">
+        <v>None specified</v>
+      </c>
+      <c r="O2" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="G2" t="str">
-        <v>The Sacred Wedding &amp; Rukhsati</v>
-      </c>
-      <c r="H2" t="str">
+      <c r="B3" t="str">
+        <v>Sep 29, 2026, 10:11 AM</v>
+      </c>
+      <c r="C3" t="str">
+        <v>as</v>
+      </c>
+      <c r="D3" t="str">
+        <v>6386687373</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Confirmed (Attending)</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3" t="str">
+        <v>⏳ Awaiting Check-In</v>
+      </c>
+      <c r="H3" t="str">
+        <v>— Not Invited</v>
+      </c>
+      <c r="I3" t="str">
+        <v>⏳ Awaiting Entry</v>
+      </c>
+      <c r="J3" t="str">
+        <v>⏳ Awaiting Entry</v>
+      </c>
+      <c r="K3" t="str">
+        <v>—</v>
+      </c>
+      <c r="L3" t="str">
+        <v>—</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Wedding Reception - Hotel Ramada; Wedding Reception - Radiant Resorts</v>
+      </c>
+      <c r="N3" t="str">
         <v>None specified</v>
       </c>
-      <c r="I2" t="str">
-        <v>Mubarak to the lovely couple!</v>
+      <c r="O3" t="str">
+        <v>fgfhghg</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sep 29, 2026, 09:56 AM</v>
+      </c>
+      <c r="C4" t="str">
+        <v>as</v>
+      </c>
+      <c r="D4" t="str">
+        <v>6386687373</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Confirmed (Attending)</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>⏳ Awaiting Check-In</v>
+      </c>
+      <c r="H4" t="str">
+        <v>— Not Invited</v>
+      </c>
+      <c r="I4" t="str">
+        <v>⏳ Awaiting Entry</v>
+      </c>
+      <c r="J4" t="str">
+        <v>⏳ Awaiting Entry</v>
+      </c>
+      <c r="K4" t="str">
+        <v>—</v>
+      </c>
+      <c r="L4" t="str">
+        <v>—</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Wedding Reception - Hotel Ramada; Wedding Reception - Radiant Resorts</v>
+      </c>
+      <c r="N4" t="str">
+        <v>None specified</v>
+      </c>
+      <c r="O4" t="str">
+        <v>fgfhghg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B15"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="45.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,47 +638,111 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Wedding Date</v>
+        <v>Sacred Rukhsati</v>
       </c>
       <c r="B3" t="str">
-        <v>Thursday, 29th October 2026</v>
+        <v>Thursday, 29th October 2026 (Shimla Resort)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Total RSVP Responses</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
+        <v>Wedding Reception 1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Friday, 30th October 2026 (Hotel Ramada)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Confirmed Attending Responses</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
+        <v>Wedding Reception 2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Monday, 2nd November 2026 (Radiant Resorts)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Total Guests (Heads)</v>
+        <v>Total RSVP Responses</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Confirmed Attending Responses</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Total Expected Guests (Heads)</v>
+      </c>
+      <c r="B8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Total Passes Checked In (Any Function)</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Rukhsati Guests Checked In</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Hotel Ramada Guests Checked In</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Radiant Resorts Guests Checked In</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Total Admitted Guests at Venue (Heads)</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Declined Responses</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>Last Updated</v>
       </c>
-      <c r="B7" t="str">
-        <v>2026-09-26T16:34:20.092Z</v>
+      <c r="B15" t="str">
+        <v>Sep 29, 2026, 10:21 AM</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update RSVP & Multi-Function Check-In sheet (0 RSVPs, 0 Checked-In) [Sep 29, 10:34 AM]
</commit_message>
<xml_diff>
--- a/wedding-rsvps.xlsx
+++ b/wedding-rsvps.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -469,31 +469,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sep 29, 2026, 10:18 AM</v>
+        <v>Sep 29, 2026, 10:33 AM</v>
       </c>
       <c r="C2" t="str">
-        <v>as</v>
+        <v>Registry Initialized</v>
       </c>
       <c r="D2" t="str">
-        <v>6386687373</v>
+        <v>—</v>
       </c>
       <c r="E2" t="str">
-        <v>Confirmed (Attending)</v>
+        <v>Awaiting Responses</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="str">
         <v>⏳ Awaiting Check-In</v>
       </c>
       <c r="H2" t="str">
-        <v>⏳ Awaiting Entry</v>
+        <v>—</v>
       </c>
       <c r="I2" t="str">
-        <v>⏳ Awaiting Entry</v>
+        <v>—</v>
       </c>
       <c r="J2" t="str">
-        <v>— Not Invited</v>
+        <v>—</v>
       </c>
       <c r="K2" t="str">
         <v>—</v>
@@ -502,112 +502,18 @@
         <v>—</v>
       </c>
       <c r="M2" t="str">
-        <v>Rukhsati; Wedding Reception - Hotel Ramada</v>
+        <v>—</v>
       </c>
       <c r="N2" t="str">
-        <v>None specified</v>
+        <v>—</v>
       </c>
       <c r="O2" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Sep 29, 2026, 10:11 AM</v>
-      </c>
-      <c r="C3" t="str">
-        <v>as</v>
-      </c>
-      <c r="D3" t="str">
-        <v>6386687373</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Confirmed (Attending)</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-      <c r="G3" t="str">
-        <v>⏳ Awaiting Check-In</v>
-      </c>
-      <c r="H3" t="str">
-        <v>— Not Invited</v>
-      </c>
-      <c r="I3" t="str">
-        <v>⏳ Awaiting Entry</v>
-      </c>
-      <c r="J3" t="str">
-        <v>⏳ Awaiting Entry</v>
-      </c>
-      <c r="K3" t="str">
-        <v>—</v>
-      </c>
-      <c r="L3" t="str">
-        <v>—</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Wedding Reception - Hotel Ramada; Wedding Reception - Radiant Resorts</v>
-      </c>
-      <c r="N3" t="str">
-        <v>None specified</v>
-      </c>
-      <c r="O3" t="str">
-        <v>fgfhghg</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Sep 29, 2026, 09:56 AM</v>
-      </c>
-      <c r="C4" t="str">
-        <v>as</v>
-      </c>
-      <c r="D4" t="str">
-        <v>6386687373</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Confirmed (Attending)</v>
-      </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4" t="str">
-        <v>⏳ Awaiting Check-In</v>
-      </c>
-      <c r="H4" t="str">
-        <v>— Not Invited</v>
-      </c>
-      <c r="I4" t="str">
-        <v>⏳ Awaiting Entry</v>
-      </c>
-      <c r="J4" t="str">
-        <v>⏳ Awaiting Entry</v>
-      </c>
-      <c r="K4" t="str">
-        <v>—</v>
-      </c>
-      <c r="L4" t="str">
-        <v>—</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Wedding Reception - Hotel Ramada; Wedding Reception - Radiant Resorts</v>
-      </c>
-      <c r="N4" t="str">
-        <v>None specified</v>
-      </c>
-      <c r="O4" t="str">
-        <v>fgfhghg</v>
+        <v>Welcome to Basit &amp; Ambiya Wedding RSVP Registry</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -665,7 +571,7 @@
         <v>Total RSVP Responses</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -673,7 +579,7 @@
         <v>Confirmed Attending Responses</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -681,7 +587,7 @@
         <v>Total Expected Guests (Heads)</v>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -737,7 +643,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B15" t="str">
-        <v>Sep 29, 2026, 10:21 AM</v>
+        <v>Sep 29, 2026, 10:33 AM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSVP & Multi-Function Check-In sheet (0 RSVPs, 0 Checked-In) [Sep 29, 10:39 AM]
</commit_message>
<xml_diff>
--- a/wedding-rsvps.xlsx
+++ b/wedding-rsvps.xlsx
@@ -469,7 +469,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sep 29, 2026, 10:33 AM</v>
+        <v>Sep 29, 2026, 10:39 AM</v>
       </c>
       <c r="C2" t="str">
         <v>Registry Initialized</v>
@@ -643,7 +643,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B15" t="str">
-        <v>Sep 29, 2026, 10:33 AM</v>
+        <v>Sep 29, 2026, 10:39 AM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSVP & Multi-Function Check-In sheet (0 RSVPs, 0 Checked-In) [Sep 29, 10:40 AM]
</commit_message>
<xml_diff>
--- a/wedding-rsvps.xlsx
+++ b/wedding-rsvps.xlsx
@@ -469,7 +469,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sep 29, 2026, 10:39 AM</v>
+        <v>Sep 29, 2026, 10:40 AM</v>
       </c>
       <c r="C2" t="str">
         <v>Registry Initialized</v>
@@ -643,7 +643,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B15" t="str">
-        <v>Sep 29, 2026, 10:39 AM</v>
+        <v>Sep 29, 2026, 10:40 AM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSVP & Multi-Function Check-In sheet (0 RSVPs, 0 Checked-In) [Sep 29, 10:42 AM]
</commit_message>
<xml_diff>
--- a/wedding-rsvps.xlsx
+++ b/wedding-rsvps.xlsx
@@ -469,7 +469,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sep 29, 2026, 10:40 AM</v>
+        <v>Sep 29, 2026, 10:42 AM</v>
       </c>
       <c r="C2" t="str">
         <v>Registry Initialized</v>
@@ -643,7 +643,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B15" t="str">
-        <v>Sep 29, 2026, 10:40 AM</v>
+        <v>Sep 29, 2026, 10:42 AM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSVP & Multi-Function Check-In sheet (1 RSVPs, 0 Checked-In) [Sep 29, 10:51 AM]
</commit_message>
<xml_diff>
--- a/wedding-rsvps.xlsx
+++ b/wedding-rsvps.xlsx
@@ -469,31 +469,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sep 29, 2026, 10:42 AM</v>
+        <v>Sep 29, 2026, 10:51 AM</v>
       </c>
       <c r="C2" t="str">
-        <v>Registry Initialized</v>
+        <v>cv</v>
       </c>
       <c r="D2" t="str">
-        <v>—</v>
+        <v>saa</v>
       </c>
       <c r="E2" t="str">
-        <v>Awaiting Responses</v>
+        <v>Confirmed (Attending)</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="str">
         <v>⏳ Awaiting Check-In</v>
       </c>
       <c r="H2" t="str">
-        <v>—</v>
+        <v>⏳ Awaiting Entry</v>
       </c>
       <c r="I2" t="str">
-        <v>—</v>
+        <v>⏳ Awaiting Entry</v>
       </c>
       <c r="J2" t="str">
-        <v>—</v>
+        <v>— Not Invited</v>
       </c>
       <c r="K2" t="str">
         <v>—</v>
@@ -502,13 +502,13 @@
         <v>—</v>
       </c>
       <c r="M2" t="str">
-        <v>—</v>
+        <v>Rukhsati; Wedding Reception - Hotel Ramada</v>
       </c>
       <c r="N2" t="str">
-        <v>—</v>
+        <v>None specified</v>
       </c>
       <c r="O2" t="str">
-        <v>Welcome to Basit &amp; Ambiya Wedding RSVP Registry</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +571,7 @@
         <v>Total RSVP Responses</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -579,7 +579,7 @@
         <v>Confirmed Attending Responses</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -587,7 +587,7 @@
         <v>Total Expected Guests (Heads)</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -643,7 +643,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B15" t="str">
-        <v>Sep 29, 2026, 10:42 AM</v>
+        <v>Sep 29, 2026, 10:51 AM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>